<commit_message>
Added new RDF data schemes and visual schemes for economy-table99-100, fixed XLSX spreadsheets economy-table99-100
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table100.xlsx
+++ b/sources/table_normalization/xlsx/economy-table100.xlsx
@@ -253,13 +253,13 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -568,7 +568,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>